<commit_message>
modified manual evaluation data
</commit_message>
<xml_diff>
--- a/manual_evaluation/functional_correctness.xlsx
+++ b/manual_evaluation/functional_correctness.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\functional\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AI IDE Analysis\AI-IDEs-code-analysis\manual_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" firstSheet="4" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" firstSheet="4" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="P1_CVBuilder" sheetId="1" r:id="rId1"/>
@@ -1911,7 +1911,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
-        <v>3.5</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>38</v>
@@ -1923,7 +1923,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
-        <v>4.0999999999999996</v>
+        <v>5.2</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>39</v>
@@ -1935,7 +1935,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
-        <v>4.2</v>
+        <v>5.3</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>40</v>

</xml_diff>